<commit_message>
fix(excel): separa completamente Categorias, Tags e Tema Central preservando dados do banco
</commit_message>
<xml_diff>
--- a/frontend/public/modelo_importacao_levihub.xlsx
+++ b/frontend/public/modelo_importacao_levihub.xlsx
@@ -28,7 +28,7 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
@@ -462,33 +462,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="32" customWidth="1" min="12" max="12"/>
-    <col width="35" customWidth="1" min="13" max="13"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="32" customWidth="1" min="13" max="13"/>
     <col width="35" customWidth="1" min="14" max="14"/>
+    <col width="35" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>PLANILHA MODELO DE IMPORTAÇÃO - LEVIHUB | Preencha a partir da linha 3 (você pode apagar as 2 linhas de exemplo). Campos obrigatórios: NOME DA MÚSICA e CATEGORIAS.</t>
+          <t>PLANILHA MODELO DE IMPORTAÇÃO - LEVIHUB | CATEGORIAS = grupos/situações (ex: agitadas1, lentas2, ceia, natal, pascoa). TAGS = palavras-chave da música (ex: jesus, cruz, amor). TEMA CENTRAL = palavra-resumo (ex: Alegria, Família).</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="24" customHeight="1">
+    <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>CÓD.</t>
@@ -511,50 +512,55 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
+          <t>TAGS / PALAVRAS-CHAVE (Separadas por vírgula)</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
           <t>TEMA CENTRAL</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>PRIMEIRA LINHA</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>TOM</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>1ª NOTA</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>VERSÃO P VOCAL</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>COMPASSO</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>BPM ≈</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>VERSÃO PARECIDA</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>LINK</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>CIFRA</t>
         </is>
@@ -578,55 +584,60 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Alegria, Agitada 1, Celebração</t>
+          <t>agitadas1, agitadas2</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
+          <t>alegria, coração, jesus, comunhão</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
           <t>Alegria</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>A alegria está no coração de quem já conhece a Jesus</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
         <is>
           <t>Original</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>4/4</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="L3" s="4" t="inlineStr">
         <is>
           <t>128</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="M3" s="4" t="inlineStr">
         <is>
           <t>Thalles Roberto - Ao Vivo</t>
         </is>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="N3" s="4" t="inlineStr">
         <is>
           <t>https://youtube.com</t>
         </is>
       </c>
-      <c r="N3" s="4" t="inlineStr"/>
+      <c r="O3" s="4" t="inlineStr"/>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
@@ -636,65 +647,74 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Minha Casa</t>
+          <t>A Mesa</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Soraya Moraes</t>
+          <t>Eli Soares</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Família, Adoração, Lenta 1</t>
+          <t>ceia, lentas2, missoes</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Família</t>
+          <t>pai, ceia, santa ceia, comunhão, pão, vinho</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>A bênção do Senhor está sobre mim</t>
+          <t>Comunhão</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
+          <t>Pão e vinho sobre a mesa</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
           <t>G</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>Feminino</t>
-        </is>
-      </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
           <t>4/4</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>75</t>
         </is>
       </c>
-      <c r="L4" s="4" t="inlineStr">
-        <is>
-          <t>Soraya Moraes - Minha Casa (Letra)</t>
-        </is>
-      </c>
-      <c r="M4" s="4" t="inlineStr"/>
-      <c r="N4" s="4" t="inlineStr"/>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>Eli Soares - A Mesa</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>https://youtu.be/J5eGCfe...</t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A1:O1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(ui): destaca que Tema Central e exclusivo para o Planejamento
</commit_message>
<xml_diff>
--- a/frontend/public/modelo_importacao_levihub.xlsx
+++ b/frontend/public/modelo_importacao_levihub.xlsx
@@ -470,7 +470,7 @@
     <col width="25" customWidth="1" min="3" max="3"/>
     <col width="36" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
     <col width="42" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
@@ -485,11 +485,11 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>PLANILHA MODELO DE IMPORTAÇÃO - LEVIHUB | CATEGORIAS = grupos/situações (ex: agitadas1, lentas2, ceia, natal, pascoa). TAGS = palavras-chave da música (ex: jesus, cruz, amor). TEMA CENTRAL = palavra-resumo (ex: Alegria, Família).</t>
+          <t>PLANILHA MODELO DE IMPORTAÇÃO - LEVIHUB | CATEGORIAS = grupos do repertório (agitadas1, lentas2, ceia...). TAGS = busca do Levi Roboto. TEMA CENTRAL = exclusivo para a tela de Planejamento.</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="26" customHeight="1">
+    <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>CÓD.</t>
@@ -517,7 +517,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>TEMA CENTRAL</t>
+          <t>TEMA CENTRAL (Exclusivo p/ Planejamento)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat: tornar tema central obrigatorio com seletor unico visual e atualizar modelo excel
</commit_message>
<xml_diff>
--- a/frontend/public/modelo_importacao_levihub.xlsx
+++ b/frontend/public/modelo_importacao_levihub.xlsx
@@ -485,7 +485,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>PLANILHA MODELO DE IMPORTAÇÃO - LEVIHUB | CATEGORIAS = grupos do repertório (agitadas1, lentas2, ceia...). TAGS = busca do Levi Roboto. TEMA CENTRAL = exclusivo para a tela de Planejamento.</t>
+          <t>PLANILHA MODELO DE IMPORTAÇÃO - LEVIHUB | Campos com (*) são obrigatórios p/ novas músicas: NOME DA MÚSICA *, CATEGORIAS *, TAGS * e TEMA CENTRAL (Exclusivo p/ Planejamento) *.</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>TEMA CENTRAL (Exclusivo p/ Planejamento)</t>
+          <t>TEMA CENTRAL (Exclusivo p/ Planejamento) *</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">

</xml_diff>